<commit_message>
Refined search + Month
</commit_message>
<xml_diff>
--- a/XLS/SCRAPE_EliRigobeliAI.xlsx
+++ b/XLS/SCRAPE_EliRigobeliAI.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H52"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,7 +430,7 @@
         <v>O Google fez de novo: Crie e Publique um Sistema Completo com IA (100% Grátis)</v>
       </c>
       <c r="B2">
-        <v>404848</v>
+        <v>404908</v>
       </c>
       <c r="C2" t="str" xml:space="preserve">
         <v xml:space="preserve">🏆 VOTE EM MIM NO PRÊMIO iBEST:
@@ -486,7 +486,7 @@
         <v>Curso Completo de N8N | Crie Agentes com IA</v>
       </c>
       <c r="B3">
-        <v>87369</v>
+        <v>87382</v>
       </c>
       <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">📌 HOSPEDAGEM N8N COM VPS NA HOSTINGER
@@ -545,7 +545,7 @@
         <v>Google Antigravity SEM LIMITES: como usar IA grátis sem travar</v>
       </c>
       <c r="B4">
-        <v>73060</v>
+        <v>73075</v>
       </c>
       <c r="C4" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -598,7 +598,7 @@
         <v>Automatize seu trabalho com um agente de IA (Claude Cowork | Guia Completo)</v>
       </c>
       <c r="B5">
-        <v>63133</v>
+        <v>63134</v>
       </c>
       <c r="C5" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -670,7 +670,7 @@
         <v>Substituí o Claude Design… e Não Tem Limites (Open Design)</v>
       </c>
       <c r="B7">
-        <v>59644</v>
+        <v>59671</v>
       </c>
       <c r="C7" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥SE INSCREVE AQUI:
@@ -750,7 +750,7 @@
         <v>ClawdBot (OpenClaw) é o melhor AGENTE de IA que já vimos (O Guia completo)</v>
       </c>
       <c r="B9">
-        <v>57274</v>
+        <v>57275</v>
       </c>
       <c r="C9" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -787,7 +787,7 @@
         <v>Gemini Super Gems: a nova forma do Google de CRIAR APPS interativos GRÁTIS</v>
       </c>
       <c r="B10">
-        <v>57151</v>
+        <v>57156</v>
       </c>
       <c r="C10" t="str" xml:space="preserve">
         <v xml:space="preserve">Nesse vídeo eu mostro como criar aplicações interativas com as Super Gems no Googel Gemini.
@@ -826,7 +826,7 @@
         <v>A forma MAIS FÁCIL de configurar o OpenClaw (ClawdBot) de forma “SEGURA” no PC (</v>
       </c>
       <c r="B11">
-        <v>56270</v>
+        <v>56272</v>
       </c>
       <c r="C11" t="str" xml:space="preserve">
         <v xml:space="preserve">⚠️ Aviso importante sobre segurança
@@ -883,7 +883,7 @@
         <v>Antes levava MESES, agora faço um APP Android em 5 minutos</v>
       </c>
       <c r="B12">
-        <v>55362</v>
+        <v>55376</v>
       </c>
       <c r="C12" t="str" xml:space="preserve">
         <v xml:space="preserve">🏆 VOTE EM MIM NO PRÊMIO iBEST:
@@ -956,7 +956,7 @@
         <v>Os Plugins do CLAUDE Cowork Mudam Tudo (Guia Completo)</v>
       </c>
       <c r="B14">
-        <v>47570</v>
+        <v>47571</v>
       </c>
       <c r="C14" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -1000,7 +1000,7 @@
         <v>Crie um APP completo do ZERO com IA (Antigravity + Claude Code)</v>
       </c>
       <c r="B15">
-        <v>43434</v>
+        <v>43438</v>
       </c>
       <c r="C15" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -1010,7 +1010,7 @@
 📌 HOSPEDAGEM VPS NA HOSTINGER
 → Use o CUPOM: ELIRIGOBELIAI (10% OFF)
 → https://links.elirigobeli.com/coolify
-Você precisa assistir estes vídeos 👇🏻
+Você precisa assistir estes vídeos ����🏻
 Antigravity: https://youtu.be/JsrsR1K2e_Y
 CLI: https://youtu.be/wbkhrHKeHnQ
 Crie Apps: https://youtu.be/JEESRkJ0fXA
@@ -1039,7 +1039,7 @@
         <v>Você Precisa Desse Agente de IA AGORA! (Adeus OpenClaw)</v>
       </c>
       <c r="B16">
-        <v>37351</v>
+        <v>37363</v>
       </c>
       <c r="C16" t="str" xml:space="preserve">
         <v xml:space="preserve">🏆 VOTE EM MIM NO PRÊMIO iBEST:
@@ -1092,7 +1092,7 @@
         <v>Novo n8n MCP: A Forma MAIS FÁCIL de Criar Apps com IA</v>
       </c>
       <c r="B17">
-        <v>35532</v>
+        <v>35534</v>
       </c>
       <c r="C17" t="str" xml:space="preserve">
         <v xml:space="preserve">Aprenda passo a passo a conectar o Claude, ChatGPT e Lovable no seu N8N usando o Novo MCP.
@@ -1165,7 +1165,7 @@
         <v>Claude mudou TUDO sobre criar agentes de IA (Managed Agents)</v>
       </c>
       <c r="B19">
-        <v>32548</v>
+        <v>32549</v>
       </c>
       <c r="C19" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -1282,7 +1282,7 @@
         <v>Agente de código 100% grátis, sem assinatura e sem API key</v>
       </c>
       <c r="B22">
-        <v>28498</v>
+        <v>28520</v>
       </c>
       <c r="C22" t="str" xml:space="preserve">
         <v xml:space="preserve">📌 HOSPEDAGEM VPS NA HOSTINGER
@@ -1364,7 +1364,7 @@
         <v>O Fable 5 FINALMENTE voltou (e você tem 7 dias)</v>
       </c>
       <c r="B24">
-        <v>26199</v>
+        <v>26211</v>
       </c>
       <c r="C24" t="str" xml:space="preserve">
         <v xml:space="preserve">🏆 VOTE EM MIM NO PRÊMIO iBEST:
@@ -1605,7 +1605,7 @@
         <v>Os Plugins do CODEX Mudam Tudo (Veja Como Usar)</v>
       </c>
       <c r="B30">
-        <v>20019</v>
+        <v>20025</v>
       </c>
       <c r="C30" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -1726,7 +1726,7 @@
         <v>A OpenAI colocou Subagentes no Codex (isso muda tudo)</v>
       </c>
       <c r="B33">
-        <v>18259</v>
+        <v>18261</v>
       </c>
       <c r="C33" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥Se inscreva para receber novidades:
@@ -1804,7 +1804,7 @@
         <v>Google ACABOU com Codex e Claude Code? Gemini 3.5 e Antigravity 2.0</v>
       </c>
       <c r="B35">
-        <v>14689</v>
+        <v>14691</v>
       </c>
       <c r="C35" t="str" xml:space="preserve">
         <v xml:space="preserve">🔥SE INSCREVE AQUI:
@@ -1831,7 +1831,7 @@
         <v>A criação de APPs com IA mudou para sempre</v>
       </c>
       <c r="B36">
-        <v>14356</v>
+        <v>14358</v>
       </c>
       <c r="C36" t="str" xml:space="preserve">
         <v xml:space="preserve">CRIE SUA CONTA:
@@ -2115,7 +2115,7 @@
         <v>O Tradutor Universal do Google chegou? A semana mais INSANA DA IA</v>
       </c>
       <c r="B43">
-        <v>11829</v>
+        <v>11831</v>
       </c>
       <c r="C43" t="str" xml:space="preserve">
         <v xml:space="preserve">Essa semana a Inteligência Artificial explodiu de novidades, e a primeira delas já levanta uma pergunta importante: a IA acabou com a barreira do idioma? Conheça o tradutor Universal do Google e outras novidades como:
@@ -2215,7 +2215,7 @@
         <v>Responda comentários do Instagram no automático (N8N)</v>
       </c>
       <c r="B45">
-        <v>10996</v>
+        <v>11004</v>
       </c>
       <c r="C45" t="str" xml:space="preserve">
         <v xml:space="preserve">📌 HOSPEDAGEM N8N COM VPS NA HOSTINGER
@@ -2305,7 +2305,7 @@
         <v>O Jeito Preguiçoso de Fazer Dinheiro com IA (2026)</v>
       </c>
       <c r="B47">
-        <v>8053</v>
+        <v>8088</v>
       </c>
       <c r="C47" t="str" xml:space="preserve">
         <v xml:space="preserve">🏆 VOTE EM MIM NO PRÊMIO iBEST:
@@ -2381,7 +2381,7 @@
         <v>Crie e PUBLIQUE seu próprio JOGO com IA (Tutorial Completo)</v>
       </c>
       <c r="B49">
-        <v>7493</v>
+        <v>7497</v>
       </c>
       <c r="C49" t="str" xml:space="preserve">
         <v xml:space="preserve">🏆 VOTE EM MIM NO PRÊMIO iBEST:
@@ -2520,85 +2520,33 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>AUTOMAÇÃO + IA - Obrigado! 10 mil inscritos</v>
+        <v>Quando as pessoas descobrirem que IA vai além do chat, o mundo conhecerá quem sa</v>
       </c>
       <c r="B52">
-        <v>2910</v>
+        <v>1113</v>
       </c>
       <c r="C52" t="str">
-        <v>elirigobeli.com/ovo</v>
+        <v>Quando as pessoas descobrirem que IA vai além do chat, o mundo conhecerá quem saiu na frente. Eli</v>
       </c>
       <c r="D52">
-        <v>221</v>
+        <v>20</v>
       </c>
       <c r="E52" t="str">
         <v/>
       </c>
       <c r="F52" t="str">
-        <v>https://www.youtube.com/shorts/nn3RKGTt_eE</v>
-      </c>
-      <c r="G52">
-        <v>15</v>
+        <v>https://www.youtube.com/shorts/qMSJ6L36nhA</v>
+      </c>
+      <c r="G52" t="str">
+        <v/>
       </c>
       <c r="H52" t="str">
-        <v>2025-07-02T00:15:12.000Z</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>Cansado do Caos Digital</v>
-      </c>
-      <c r="B53">
-        <v>1199</v>
-      </c>
-      <c r="C53" t="str">
-        <v>LINK: https://segundocerebro.com.br/clique_...</v>
-      </c>
-      <c r="D53">
-        <v>41</v>
-      </c>
-      <c r="E53" t="str">
-        <v/>
-      </c>
-      <c r="F53" t="str">
-        <v>https://www.youtube.com/shorts/N_tVrLo0NQE</v>
-      </c>
-      <c r="G53">
-        <v>1</v>
-      </c>
-      <c r="H53" t="str">
-        <v>2024-05-10T20:45:00.000Z</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>Quando as pessoas descobrirem que IA vai além do chat, o mundo conhecerá quem sa</v>
-      </c>
-      <c r="B54">
-        <v>1113</v>
-      </c>
-      <c r="C54" t="str">
-        <v>Quando as pessoas descobrirem que IA vai além do chat, o mundo conhecerá quem saiu na frente. Eli</v>
-      </c>
-      <c r="D54">
-        <v>20</v>
-      </c>
-      <c r="E54" t="str">
-        <v/>
-      </c>
-      <c r="F54" t="str">
-        <v>https://www.youtube.com/shorts/qMSJ6L36nhA</v>
-      </c>
-      <c r="G54" t="str">
-        <v/>
-      </c>
-      <c r="H54" t="str">
         <v>2026-07-04T19:37:10.000Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H52"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>